<commit_message>
Model: capital sheet now starts from the filed 10-K number
</commit_message>
<xml_diff>
--- a/model/ALHC_model.xlsx
+++ b/model/ALHC_model.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="295">
   <si>
     <t xml:space="preserve">ALHC model inputs (blue = hardcoded input; yellow = key assumption). $ in millions unless noted.</t>
   </si>
@@ -683,7 +683,7 @@
     <t xml:space="preserve">California tangible net equity (TNE) check, Knox-Keene formula as described in the Q2 2026 10-Q, note 11</t>
   </si>
   <si>
-    <t xml:space="preserve">Required = 150% of the largest of $1m; 2% of first $150m of annualized premium + 1% above; 8% of first $150m of non-capitated health care spend + 4% above. Amounts are not disclosed; this is an outside estimate.</t>
+    <t xml:space="preserve">Required = 150% of the largest of $1m; 2% of first $150m of annualized premium + 1% above; 8% of first $150m of non-capitated health care spend + 4% above. Per-plan amounts are not disclosed. The 10-K gives the aggregate: regulatory capital $268.5m vs a $116.1m minimum at 31 Dec 2025 (data/regulatory_capital.csv).</t>
   </si>
   <si>
     <t xml:space="preserve">FY26E</t>
@@ -734,16 +734,28 @@
     <t xml:space="preserve">Max of premium test and 0%-capitated spend test</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimated regulated net worth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equity + parent debt - parent cash - goodwill/intangibles (rough)</t>
+    <t xml:space="preserve">Regulatory capital (filed YE25, plus net income)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-K FY2025: $268.5m at 31 Dec 2025, rolled forward with consolidated net income (all subsidiaries, all states)</t>
   </si>
   <si>
     <t xml:space="preserve">Headroom, low requirement</t>
   </si>
   <si>
     <t xml:space="preserve">Headroom, high requirement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum, all states, at the 2025 ratio to revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-K FY2025: $116.1m minimum on $3,948.7m revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cover vs that minimum (x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filed 2.31x at YE25 (2.08x YE24)</t>
   </si>
   <si>
     <t xml:space="preserve">Valuation: same method for any managed-care stock. Peer data Yahoo Finance, 16 Oct 2026 closes and 17 Oct consensus.</t>
@@ -903,7 +915,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="166" formatCode="#,##0.0;\(#,##0.0\);\-"/>
@@ -911,9 +923,10 @@
     <numFmt numFmtId="168" formatCode="0.00%;\(0.00%\);\-"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
     <numFmt numFmtId="170" formatCode="#,##0"/>
-    <numFmt numFmtId="171" formatCode="@"/>
-    <numFmt numFmtId="172" formatCode="#,##0.00"/>
-    <numFmt numFmtId="173" formatCode="0.0\x"/>
+    <numFmt numFmtId="171" formatCode="0.00\x"/>
+    <numFmt numFmtId="172" formatCode="@"/>
+    <numFmt numFmtId="173" formatCode="#,##0.00"/>
+    <numFmt numFmtId="174" formatCode="0.0\x"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -1020,7 +1033,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1109,11 +1122,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1121,11 +1138,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1133,7 +1150,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5830,7 +5847,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -6022,16 +6039,16 @@
         <v>236</v>
       </c>
       <c r="B12" s="17" t="n">
-        <f aca="false">Model!P42+Model!P40-Inputs!$B$39-(32.06+4.55)</f>
-        <v>433.27672</v>
+        <f aca="false">268.515+Model!P22</f>
+        <v>295.10272</v>
       </c>
       <c r="C12" s="17" t="n">
-        <f aca="false">Model!Q42+Model!Q40-Inputs!$B$39-(32.06+4.55)</f>
-        <v>587.15846628618</v>
+        <f aca="false">B12+Model!Q22</f>
+        <v>370.37366628618</v>
       </c>
       <c r="D12" s="17" t="n">
-        <f aca="false">Model!R42+Model!R40-Inputs!$B$39-(32.06+4.55)</f>
-        <v>752.788800675986</v>
+        <f aca="false">C12+Model!R22</f>
+        <v>453.576660675986</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>237</v>
@@ -6043,15 +6060,15 @@
       </c>
       <c r="B13" s="17" t="n">
         <f aca="false">B12-B10</f>
-        <v>317.133121048</v>
+        <v>178.959121048</v>
       </c>
       <c r="C13" s="17" t="n">
         <f aca="false">C12-C10</f>
-        <v>445.08031431755</v>
+        <v>228.29551431755</v>
       </c>
       <c r="D13" s="17" t="n">
         <f aca="false">D12-D10</f>
-        <v>585.714806835814</v>
+        <v>286.502666835814</v>
       </c>
       <c r="E13" s="4"/>
     </row>
@@ -6061,17 +6078,57 @@
       </c>
       <c r="B14" s="17" t="n">
         <f aca="false">B12-B11</f>
-        <v>209.989522096</v>
+        <v>71.815522096</v>
       </c>
       <c r="C14" s="17" t="n">
         <f aca="false">C12-C11</f>
-        <v>312.00216234892</v>
+        <v>95.21736234892</v>
       </c>
       <c r="D14" s="17" t="n">
         <f aca="false">D12-D11</f>
-        <v>427.640812995641</v>
+        <v>128.428672995642</v>
       </c>
       <c r="E14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <f aca="false">116.09/3948.719*Model!P8</f>
+        <v>153.170914415536</v>
+      </c>
+      <c r="C15" s="17" t="n">
+        <f aca="false">116.09/3948.719*Model!Q8</f>
+        <v>190.375310064681</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <f aca="false">116.09/3948.719*Model!R8</f>
+        <v>226.134824434789</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B16" s="21" t="n">
+        <f aca="false">B12/B15</f>
+        <v>1.92662374006216</v>
+      </c>
+      <c r="C16" s="21" t="n">
+        <f aca="false">C12/C15</f>
+        <v>1.94549212374412</v>
+      </c>
+      <c r="D16" s="21" t="n">
+        <f aca="false">D12/D15</f>
+        <v>2.00577979004195</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>243</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6098,7 +6155,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6130,370 +6187,370 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
-        <v>254</v>
-      </c>
-      <c r="B4" s="22" t="n">
+      <c r="A4" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="B4" s="23" t="n">
         <v>401.43</v>
       </c>
-      <c r="C4" s="22" t="n">
+      <c r="C4" s="23" t="n">
         <v>383.55</v>
       </c>
-      <c r="D4" s="22" t="n">
+      <c r="D4" s="23" t="n">
         <v>897.594847</v>
       </c>
-      <c r="E4" s="22" t="n">
+      <c r="E4" s="23" t="n">
         <v>409287.852032</v>
       </c>
-      <c r="F4" s="22" t="n">
+      <c r="F4" s="23" t="n">
         <v>28903.000064</v>
       </c>
-      <c r="G4" s="22" t="n">
+      <c r="G4" s="23" t="n">
         <v>20.51338</v>
       </c>
-      <c r="H4" s="22" t="n">
+      <c r="H4" s="23" t="n">
         <v>23.22918</v>
       </c>
-      <c r="I4" s="23" t="n">
+      <c r="I4" s="24" t="n">
         <f aca="false">B4/H4</f>
         <v>17.28128156052</v>
       </c>
-      <c r="J4" s="24" t="n">
+      <c r="J4" s="25" t="n">
         <f aca="false">F4+(H4-G4)*D4/(1-Inputs!$B$32)</f>
         <v>32110.4843870034</v>
       </c>
-      <c r="K4" s="23" t="n">
+      <c r="K4" s="24" t="n">
         <f aca="false">E4/J4</f>
         <v>12.7462372444826</v>
       </c>
-      <c r="L4" s="23" t="n">
+      <c r="L4" s="24" t="n">
         <f aca="false">C4/H4</f>
         <v>16.5115600292391</v>
       </c>
-      <c r="M4" s="23" t="n">
+      <c r="M4" s="24" t="n">
         <f aca="false">(E4+(C4-B4)*D4)/J4</f>
         <v>12.2464317706401</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
-        <v>255</v>
-      </c>
-      <c r="B5" s="22" t="n">
+      <c r="A5" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="B5" s="23" t="n">
         <v>413.16</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="23" t="n">
         <v>407.02</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="23" t="n">
         <v>120.080308</v>
       </c>
-      <c r="E5" s="22" t="n">
+      <c r="E5" s="23" t="n">
         <v>40549.380096</v>
       </c>
-      <c r="F5" s="22" t="n">
+      <c r="F5" s="23" t="n">
         <v>3596</v>
       </c>
-      <c r="G5" s="22" t="n">
+      <c r="G5" s="23" t="n">
         <v>9.15913</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="23" t="n">
         <v>17.08832</v>
       </c>
-      <c r="I5" s="23" t="n">
+      <c r="I5" s="24" t="n">
         <f aca="false">B5/H5</f>
         <v>24.1779180165165</v>
       </c>
-      <c r="J5" s="24" t="n">
+      <c r="J5" s="25" t="n">
         <f aca="false">F5+(H5-G5)*D5/(1-Inputs!$B$32)</f>
         <v>4848.81523340858</v>
       </c>
-      <c r="K5" s="23" t="n">
+      <c r="K5" s="24" t="n">
         <f aca="false">E5/J5</f>
         <v>8.36273979190066</v>
       </c>
-      <c r="L5" s="23" t="n">
+      <c r="L5" s="24" t="n">
         <f aca="false">C5/H5</f>
         <v>23.8186082657628</v>
       </c>
-      <c r="M5" s="23" t="n">
+      <c r="M5" s="24" t="n">
         <f aca="false">(E5+(C5-B5)*D5)/J5</f>
         <v>8.21068345326354</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
-        <v>256</v>
-      </c>
-      <c r="B6" s="22" t="n">
+      <c r="A6" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="B6" s="23" t="n">
         <v>428.26</v>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="23" t="n">
         <v>424.24</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="23" t="n">
         <v>216.86929</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="23" t="n">
         <v>86545.440768</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="23" t="n">
         <v>8323.999744</v>
       </c>
-      <c r="G6" s="22" t="n">
+      <c r="G6" s="23" t="n">
         <v>27.24418</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="23" t="n">
         <v>29.60006</v>
       </c>
-      <c r="I6" s="23" t="n">
+      <c r="I6" s="24" t="n">
         <f aca="false">B6/H6</f>
         <v>14.4682139157826</v>
       </c>
-      <c r="J6" s="24" t="n">
+      <c r="J6" s="25" t="n">
         <f aca="false">F6+(H6-G6)*D6/(1-Inputs!$B$32)</f>
         <v>8996.26030048053</v>
       </c>
-      <c r="K6" s="23" t="n">
+      <c r="K6" s="24" t="n">
         <f aca="false">E6/J6</f>
         <v>9.62015747403143</v>
       </c>
-      <c r="L6" s="23" t="n">
+      <c r="L6" s="24" t="n">
         <f aca="false">C6/H6</f>
         <v>14.3324033802634</v>
       </c>
-      <c r="M6" s="23" t="n">
+      <c r="M6" s="24" t="n">
         <f aca="false">(E6+(C6-B6)*D6)/J6</f>
         <v>9.52324892351368</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>257</v>
-      </c>
-      <c r="B7" s="22" t="n">
+      <c r="A7" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="B7" s="23" t="n">
         <v>92.36</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>95.55</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>1278.970369</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="23" t="n">
         <v>180670.70976</v>
       </c>
-      <c r="F7" s="22" t="n">
+      <c r="F7" s="23" t="n">
         <v>16679.999488</v>
       </c>
-      <c r="G7" s="22" t="n">
+      <c r="G7" s="23" t="n">
         <v>8.04287</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="23" t="n">
         <v>8.53519</v>
       </c>
-      <c r="I7" s="23" t="n">
+      <c r="I7" s="24" t="n">
         <f aca="false">B7/H7</f>
         <v>10.8210830690354</v>
       </c>
-      <c r="J7" s="24" t="n">
+      <c r="J7" s="25" t="n">
         <f aca="false">F7+(H7-G7)*D7/(1-Inputs!$B$32)</f>
         <v>17508.5030301922</v>
       </c>
-      <c r="K7" s="23" t="n">
+      <c r="K7" s="24" t="n">
         <f aca="false">E7/J7</f>
         <v>10.3190266722658</v>
       </c>
-      <c r="L7" s="23" t="n">
+      <c r="L7" s="24" t="n">
         <f aca="false">C7/H7</f>
         <v>11.1948298749061</v>
       </c>
-      <c r="M7" s="23" t="n">
+      <c r="M7" s="24" t="n">
         <f aca="false">(E7+(C7-B7)*D7)/J7</f>
         <v>10.5520514757041</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
-        <v>258</v>
-      </c>
-      <c r="B8" s="22" t="n">
+      <c r="A8" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="B8" s="23" t="n">
         <v>69.16</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>69.41</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="23" t="n">
         <v>493.995</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="23" t="n">
         <v>23307.69408</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="23" t="n">
         <v>4606.000128</v>
       </c>
-      <c r="G8" s="22" t="n">
+      <c r="G8" s="23" t="n">
         <v>4.88462</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="23" t="n">
         <v>5.34776</v>
       </c>
-      <c r="I8" s="23" t="n">
+      <c r="I8" s="24" t="n">
         <f aca="false">B8/H8</f>
         <v>12.9325175400542</v>
       </c>
-      <c r="J8" s="24" t="n">
+      <c r="J8" s="25" t="n">
         <f aca="false">F8+(H8-G8)*D8/(1-Inputs!$B$32)</f>
         <v>4907.03808102632</v>
       </c>
-      <c r="K8" s="23" t="n">
+      <c r="K8" s="24" t="n">
         <f aca="false">E8/J8</f>
         <v>4.74984984732891</v>
       </c>
-      <c r="L8" s="23" t="n">
+      <c r="L8" s="24" t="n">
         <f aca="false">C8/H8</f>
         <v>12.9792660852394</v>
       </c>
-      <c r="M8" s="23" t="n">
+      <c r="M8" s="24" t="n">
         <f aca="false">(E8+(C8-B8)*D8)/J8</f>
         <v>4.775017524441</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>259</v>
-      </c>
-      <c r="B9" s="22" t="n">
+      <c r="A9" s="22" t="s">
+        <v>263</v>
+      </c>
+      <c r="B9" s="23" t="n">
         <v>207.36</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <v>214.07</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="23" t="n">
         <v>52.2</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="23" t="n">
         <v>5862.192128</v>
       </c>
-      <c r="F9" s="22" t="n">
+      <c r="F9" s="23" t="n">
         <v>390</v>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="G9" s="23" t="n">
         <v>5.24983</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="23" t="n">
         <v>8.55097</v>
       </c>
-      <c r="I9" s="23" t="n">
+      <c r="I9" s="24" t="n">
         <f aca="false">B9/H9</f>
         <v>24.2498804229228</v>
       </c>
-      <c r="J9" s="24" t="n">
+      <c r="J9" s="25" t="n">
         <f aca="false">F9+(H9-G9)*D9/(1-Inputs!$B$32)</f>
         <v>616.736194736842</v>
       </c>
-      <c r="K9" s="23" t="n">
+      <c r="K9" s="24" t="n">
         <f aca="false">E9/J9</f>
         <v>9.50518581206567</v>
       </c>
-      <c r="L9" s="23" t="n">
+      <c r="L9" s="24" t="n">
         <f aca="false">C9/H9</f>
         <v>25.0345867194014</v>
       </c>
-      <c r="M9" s="23" t="n">
+      <c r="M9" s="24" t="n">
         <f aca="false">(E9+(C9-B9)*D9)/J9</f>
         <v>10.0731142115809</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>260</v>
-      </c>
-      <c r="B10" s="22" t="n">
+      <c r="A10" s="22" t="s">
+        <v>264</v>
+      </c>
+      <c r="B10" s="23" t="n">
         <v>302.3</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>290.05</v>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="D10" s="23" t="n">
         <v>264.240486</v>
       </c>
-      <c r="E10" s="22" t="n">
+      <c r="E10" s="23" t="n">
         <v>104790.900736</v>
       </c>
-      <c r="F10" s="22" t="n">
+      <c r="F10" s="23" t="n">
         <v>12757.999616</v>
       </c>
-      <c r="G10" s="22" t="n">
+      <c r="G10" s="23" t="n">
         <v>30.51015</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="23" t="n">
         <v>33.48462</v>
       </c>
-      <c r="I10" s="23" t="n">
+      <c r="I10" s="24" t="n">
         <f aca="false">B10/H10</f>
         <v>9.02802540390185</v>
       </c>
-      <c r="J10" s="24" t="n">
+      <c r="J10" s="25" t="n">
         <f aca="false">F10+(H10-G10)*D10/(1-Inputs!$B$32)</f>
         <v>13792.1777717795</v>
       </c>
-      <c r="K10" s="23" t="n">
+      <c r="K10" s="24" t="n">
         <f aca="false">E10/J10</f>
         <v>7.59785020683355</v>
       </c>
-      <c r="L10" s="23" t="n">
+      <c r="L10" s="24" t="n">
         <f aca="false">C10/H10</f>
         <v>8.66218580351218</v>
       </c>
-      <c r="M10" s="23" t="n">
+      <c r="M10" s="24" t="n">
         <f aca="false">(E10+(C10-B10)*D10)/J10</f>
         <v>7.36315587450533</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -6502,27 +6559,27 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="25" t="n">
+      <c r="I11" s="26" t="n">
         <f aca="false">MEDIAN(I4:I10)</f>
         <v>14.4682139157826</v>
       </c>
       <c r="J11" s="2"/>
-      <c r="K11" s="25" t="n">
+      <c r="K11" s="26" t="n">
         <f aca="false">MEDIAN(K4:K10)</f>
         <v>9.50518581206567</v>
       </c>
-      <c r="L11" s="25" t="n">
+      <c r="L11" s="26" t="n">
         <f aca="false">MEDIAN(L4:L10)</f>
         <v>14.3324033802634</v>
       </c>
-      <c r="M11" s="25" t="n">
+      <c r="M11" s="26" t="n">
         <f aca="false">MEDIAN(M4:M10)</f>
         <v>9.52324892351368</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -6531,27 +6588,27 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="23" t="n">
+      <c r="I12" s="24" t="n">
         <f aca="false">MEDIAN(I4,I6,I7,I8,I10)</f>
         <v>12.9325175400542</v>
       </c>
       <c r="J12" s="2"/>
-      <c r="K12" s="23" t="n">
+      <c r="K12" s="24" t="n">
         <f aca="false">MEDIAN(K4,K6,K7,K8,K10)</f>
         <v>9.62015747403143</v>
       </c>
-      <c r="L12" s="23" t="n">
+      <c r="L12" s="24" t="n">
         <f aca="false">MEDIAN(L4,L6,L7,L8,L10)</f>
         <v>12.9792660852394</v>
       </c>
-      <c r="M12" s="23" t="n">
+      <c r="M12" s="24" t="n">
         <f aca="false">MEDIAN(M4,M6,M7,M8,M10)</f>
         <v>9.52324892351368</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -6583,7 +6640,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -6600,7 +6657,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">Model!Q8</f>
@@ -6640,7 +6697,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B18" s="16" t="n">
         <f aca="false">Inputs!$B$23</f>
@@ -6660,7 +6717,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B19" s="17" t="n">
         <f aca="false">Model!Q16</f>
@@ -6680,7 +6737,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B20" s="17" t="n">
         <f aca="false">Model!Q17+Model!Q18</f>
@@ -6700,7 +6757,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">Model!Q23</f>
@@ -6720,7 +6777,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B22" s="17" t="n">
         <f aca="false">Model!Q24</f>
@@ -6740,9 +6797,9 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="B23" s="26" t="n">
+        <v>275</v>
+      </c>
+      <c r="B23" s="27" t="n">
         <f aca="false">I11</f>
         <v>14.4682139157826</v>
       </c>
@@ -6760,9 +6817,9 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="B24" s="26" t="n">
+        <v>276</v>
+      </c>
+      <c r="B24" s="27" t="n">
         <f aca="false">K11</f>
         <v>9.50518581206567</v>
       </c>
@@ -6780,7 +6837,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B25" s="19" t="n">
         <f aca="false">Inputs!$B$42*0.21*Inputs!$B$43/B22</f>
@@ -6800,7 +6857,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B26" s="17" t="n">
         <f aca="false">Inputs!$B$41-Inputs!$B$39</f>
@@ -6820,7 +6877,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B27" s="19" t="n">
         <f aca="false">B23*B21*(1-Inputs!$B$32)/B22+B25</f>
@@ -6840,7 +6897,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="B28" s="19" t="n">
         <f aca="false">(B24*B19-B26)/B22</f>
@@ -6860,7 +6917,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="B29" s="19" t="n">
         <f aca="false">-Inputs!$B$27</f>
@@ -6880,7 +6937,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B30" s="18" t="n">
         <f aca="false">AVERAGE(B27,B28)+B29</f>
@@ -6900,7 +6957,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="B31" s="16" t="n">
         <f aca="false">B30/Inputs!$B$4-1</f>
@@ -6935,7 +6992,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -6952,9 +7009,9 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="B34" s="27" t="n">
+        <v>285</v>
+      </c>
+      <c r="B34" s="28" t="n">
         <f aca="false">1-B18-((2*(Inputs!$B$4+Inputs!$B$27)-B25+I11*B20*(1-Inputs!$B$32)/B22+B26/B22)/(I11*(1-Inputs!$B$32)/B22+K11/B22))/B16</f>
         <v>0.874353226788067</v>
       </c>
@@ -6972,9 +7029,9 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>282</v>
-      </c>
-      <c r="B35" s="27" t="n">
+        <v>286</v>
+      </c>
+      <c r="B35" s="28" t="n">
         <f aca="false">1-B18-((2*(Inputs!$B$5+0.31*Inputs!$B$27)-B25+L11*B20*(1-Inputs!$B$32)/B22+B26/B22)/(L11*(1-Inputs!$B$32)/B22+M11/B22))/B16</f>
         <v>0.860832755254102</v>
       </c>
@@ -6992,9 +7049,9 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="B36" s="27" t="n">
+        <v>287</v>
+      </c>
+      <c r="B36" s="28" t="n">
         <f aca="false">B34-B35</f>
         <v>0.0135204715339643</v>
       </c>
@@ -7042,7 +7099,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -7085,30 +7142,30 @@
       <c r="M40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="28" t="n">
+      <c r="A41" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="B41" s="29" t="n">
+      <c r="B41" s="30" t="n">
         <f aca="false">AVERAGE($A41*(($B$16*(1-B$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-B$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>8.70764624452213</v>
       </c>
-      <c r="C41" s="29" t="n">
+      <c r="C41" s="30" t="n">
         <f aca="false">AVERAGE($A41*(($B$16*(1-C$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-C$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>7.34266997341081</v>
       </c>
-      <c r="D41" s="29" t="n">
+      <c r="D41" s="30" t="n">
         <f aca="false">AVERAGE($A41*(($B$16*(1-D$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-D$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>6.25068895652175</v>
       </c>
-      <c r="E41" s="29" t="n">
+      <c r="E41" s="30" t="n">
         <f aca="false">AVERAGE($A41*(($B$16*(1-E$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-E$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>4.61271743118816</v>
       </c>
-      <c r="F41" s="29" t="n">
+      <c r="F41" s="30" t="n">
         <f aca="false">AVERAGE($A41*(($B$16*(1-F$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-F$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>3.24774116007684</v>
       </c>
-      <c r="G41" s="29" t="n">
+      <c r="G41" s="30" t="n">
         <f aca="false">AVERAGE($A41*(($B$16*(1-G$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-G$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>1.88276488896552</v>
       </c>
@@ -7120,30 +7177,30 @@
       <c r="M41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="28" t="n">
+      <c r="A42" s="29" t="n">
         <v>13</v>
       </c>
-      <c r="B42" s="29" t="n">
+      <c r="B42" s="30" t="n">
         <f aca="false">AVERAGE($A42*(($B$16*(1-B$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-B$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>9.06436378349104</v>
       </c>
-      <c r="C42" s="29" t="n">
+      <c r="C42" s="30" t="n">
         <f aca="false">AVERAGE($A42*(($B$16*(1-C$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-C$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>7.64368970745513</v>
       </c>
-      <c r="D42" s="29" t="n">
+      <c r="D42" s="30" t="n">
         <f aca="false">AVERAGE($A42*(($B$16*(1-D$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-D$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>6.5071504466264</v>
       </c>
-      <c r="E42" s="29" t="n">
+      <c r="E42" s="30" t="n">
         <f aca="false">AVERAGE($A42*(($B$16*(1-E$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-E$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>4.80234155538331</v>
       </c>
-      <c r="F42" s="29" t="n">
+      <c r="F42" s="30" t="n">
         <f aca="false">AVERAGE($A42*(($B$16*(1-F$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-F$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>3.3816674793474</v>
       </c>
-      <c r="G42" s="29" t="n">
+      <c r="G42" s="30" t="n">
         <f aca="false">AVERAGE($A42*(($B$16*(1-G$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-G$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>1.9609934033115</v>
       </c>
@@ -7155,30 +7212,30 @@
       <c r="M42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="28" t="n">
+      <c r="A43" s="29" t="n">
         <v>14.5</v>
       </c>
-      <c r="B43" s="29" t="n">
+      <c r="B43" s="30" t="n">
         <f aca="false">AVERAGE($A43*(($B$16*(1-B$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-B$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>9.5994400919444</v>
       </c>
-      <c r="C43" s="29" t="n">
+      <c r="C43" s="30" t="n">
         <f aca="false">AVERAGE($A43*(($B$16*(1-C$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-C$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>8.09521930852161</v>
       </c>
-      <c r="D43" s="29" t="n">
+      <c r="D43" s="30" t="n">
         <f aca="false">AVERAGE($A43*(($B$16*(1-D$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-D$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>6.89184268178338</v>
       </c>
-      <c r="E43" s="29" t="n">
+      <c r="E43" s="30" t="n">
         <f aca="false">AVERAGE($A43*(($B$16*(1-E$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-E$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>5.08677774167604</v>
       </c>
-      <c r="F43" s="29" t="n">
+      <c r="F43" s="30" t="n">
         <f aca="false">AVERAGE($A43*(($B$16*(1-F$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-F$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>3.58255695825325</v>
       </c>
-      <c r="G43" s="29" t="n">
+      <c r="G43" s="30" t="n">
         <f aca="false">AVERAGE($A43*(($B$16*(1-G$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-G$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>2.07833617483046</v>
       </c>
@@ -7190,30 +7247,30 @@
       <c r="M43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="28" t="n">
+      <c r="A44" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="B44" s="29" t="n">
+      <c r="B44" s="30" t="n">
         <f aca="false">AVERAGE($A44*(($B$16*(1-B$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-B$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>10.1345164003978</v>
       </c>
-      <c r="C44" s="29" t="n">
+      <c r="C44" s="30" t="n">
         <f aca="false">AVERAGE($A44*(($B$16*(1-C$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-C$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>8.5467489095881</v>
       </c>
-      <c r="D44" s="29" t="n">
+      <c r="D44" s="30" t="n">
         <f aca="false">AVERAGE($A44*(($B$16*(1-D$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-D$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>7.27653491694036</v>
       </c>
-      <c r="E44" s="29" t="n">
+      <c r="E44" s="30" t="n">
         <f aca="false">AVERAGE($A44*(($B$16*(1-E$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-E$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>5.37121392796876</v>
       </c>
-      <c r="F44" s="29" t="n">
+      <c r="F44" s="30" t="n">
         <f aca="false">AVERAGE($A44*(($B$16*(1-F$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-F$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>3.78344643715909</v>
       </c>
-      <c r="G44" s="29" t="n">
+      <c r="G44" s="30" t="n">
         <f aca="false">AVERAGE($A44*(($B$16*(1-G$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-G$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>2.19567894634942</v>
       </c>
@@ -7225,30 +7282,30 @@
       <c r="M44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="28" t="n">
+      <c r="A45" s="29" t="n">
         <v>17</v>
       </c>
-      <c r="B45" s="29" t="n">
+      <c r="B45" s="30" t="n">
         <f aca="false">AVERAGE($A45*(($B$16*(1-B$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-B$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>10.4912339393667</v>
       </c>
-      <c r="C45" s="29" t="n">
+      <c r="C45" s="30" t="n">
         <f aca="false">AVERAGE($A45*(($B$16*(1-C$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-C$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>8.84776864363242</v>
       </c>
-      <c r="D45" s="29" t="n">
+      <c r="D45" s="30" t="n">
         <f aca="false">AVERAGE($A45*(($B$16*(1-D$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-D$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>7.53299640704501</v>
       </c>
-      <c r="E45" s="29" t="n">
+      <c r="E45" s="30" t="n">
         <f aca="false">AVERAGE($A45*(($B$16*(1-E$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-E$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>5.56083805216391</v>
       </c>
-      <c r="F45" s="29" t="n">
+      <c r="F45" s="30" t="n">
         <f aca="false">AVERAGE($A45*(($B$16*(1-F$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-F$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>3.91737275642965</v>
       </c>
-      <c r="G45" s="29" t="n">
+      <c r="G45" s="30" t="n">
         <f aca="false">AVERAGE($A45*(($B$16*(1-G$40-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($K$11*($B$16*(1-G$40-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>2.2739074606954</v>
       </c>
@@ -7291,7 +7348,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -7308,19 +7365,19 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
@@ -7335,7 +7392,7 @@
       <c r="A50" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B50" s="27" t="n">
+      <c r="B50" s="28" t="n">
         <f aca="false">'MBR Bridge'!B12</f>
         <v>0.893442080794731</v>
       </c>
@@ -7343,11 +7400,11 @@
         <f aca="false">($B$16*(1-B50-$B$18))</f>
         <v>107.220493308961</v>
       </c>
-      <c r="D50" s="29" t="n">
+      <c r="D50" s="30" t="n">
         <f aca="false">(($B$16*(1-B50-$B$18))-$B$20)/$B$22</f>
         <v>0.251534343006963</v>
       </c>
-      <c r="E50" s="29" t="n">
+      <c r="E50" s="30" t="n">
         <f aca="false">AVERAGE($B$23*(($B$16*(1-B50-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($B$24*($B$16*(1-B50-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>2.54398885343439</v>
       </c>
@@ -7364,7 +7421,7 @@
       <c r="A51" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B51" s="27" t="n">
+      <c r="B51" s="28" t="n">
         <f aca="false">'MBR Bridge'!C12</f>
         <v>0.878107152152697</v>
       </c>
@@ -7372,11 +7429,11 @@
         <f aca="false">($B$16*(1-B51-$B$18))</f>
         <v>206.521534307718</v>
       </c>
-      <c r="D51" s="29" t="n">
+      <c r="D51" s="30" t="n">
         <f aca="false">(($B$16*(1-B51-$B$18))-$B$20)/$B$22</f>
         <v>0.701072166184034</v>
       </c>
-      <c r="E51" s="29" t="n">
+      <c r="E51" s="30" t="n">
         <f aca="false">AVERAGE($B$23*(($B$16*(1-B51-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($B$24*($B$16*(1-B51-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>7.1519826906644</v>
       </c>
@@ -7393,7 +7450,7 @@
       <c r="A52" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B52" s="27" t="n">
+      <c r="B52" s="28" t="n">
         <f aca="false">'MBR Bridge'!D12</f>
         <v>0.869795155888973</v>
       </c>
@@ -7401,11 +7458,11 @@
         <f aca="false">($B$16*(1-B52-$B$18))</f>
         <v>260.345709237573</v>
       </c>
-      <c r="D52" s="29" t="n">
+      <c r="D52" s="30" t="n">
         <f aca="false">(($B$16*(1-B52-$B$18))-$B$20)/$B$22</f>
         <v>0.944735295884472</v>
       </c>
-      <c r="E52" s="29" t="n">
+      <c r="E52" s="30" t="n">
         <f aca="false">AVERAGE($B$23*(($B$16*(1-B52-$B$18))-$B$20)*(1-Inputs!$B$32)/$B$22+$B$25,($B$24*($B$16*(1-B52-$B$18))-$B$26)/$B$22)-Inputs!$B$27</f>
         <v>9.64965506022058</v>
       </c>

</xml_diff>